<commit_message>
Tappa Zero: toglie la sezione «chi fa cosa»
Via la pagina dal PDF (ora 14 pagine) e il conteggio per persona dal foglio
Attività dell'Excel. I responsabili restano indicati su ogni attività.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNYo6uPPTyzbFJvdbw6
</commit_message>
<xml_diff>
--- a/piano-tappa-zero-2026/dist/piano-tappa-zero-2026.xlsx
+++ b/piano-tappa-zero-2026/dist/piano-tappa-zero-2026.xlsx
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="271">
   <si>
     <t xml:space="preserve">PIANO OPERATIVO · TAPPA ZERO</t>
   </si>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">Timeline operativa delle 2 giornate</t>
   </si>
   <si>
-    <t xml:space="preserve">Chi fa cosa e quando, per lo staff operativo.</t>
+    <t xml:space="preserve">Orari, ruoli e passaggi delle due giornate per lo staff operativo.</t>
   </si>
   <si>
     <t xml:space="preserve">mezza giornata</t>
@@ -402,24 +402,6 @@
   </si>
   <si>
     <t xml:space="preserve">Alberto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHI FA COSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N. attività</t>
-  </si>
-  <si>
-    <t xml:space="preserve">di cui P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stefano Cagnoni</t>
   </si>
   <si>
     <t xml:space="preserve">PREVENTIVO DI SPESA · TAPPA ZERO</t>
@@ -988,15 +970,15 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="167" formatCode="General"/>
-    <numFmt numFmtId="168" formatCode="&quot;€ &quot;#,##0.00;&quot;-€ &quot;#,##0.00;\–"/>
-    <numFmt numFmtId="169" formatCode="#,##0"/>
-    <numFmt numFmtId="170" formatCode="&quot;€ &quot;#,##0.00##;&quot;-€ &quot;#,##0.00##;\–"/>
+    <numFmt numFmtId="167" formatCode="&quot;€ &quot;#,##0.00;&quot;-€ &quot;#,##0.00;\–"/>
+    <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="&quot;€ &quot;#,##0.00##;&quot;-€ &quot;#,##0.00##;\–"/>
+    <numFmt numFmtId="170" formatCode="General"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
     <numFmt numFmtId="172" formatCode="0%"/>
     <numFmt numFmtId="173" formatCode="&quot;€ &quot;#,##0"/>
   </numFmts>
-  <fonts count="47">
+  <fonts count="44">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,30 +1151,6 @@
     <font>
       <sz val="9"/>
       <color rgb="FF3A403A"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF0072CE"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF6B706B"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF0A0C0A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1473,8 +1431,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color rgb="FFD5DAD5"/>
+      <bottom style="medium">
+        <color rgb="FFB7791F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1482,8 +1440,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color rgb="FFB7791F"/>
+      <bottom style="thin">
+        <color rgb="FFD5DAD5"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1522,7 +1480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="77">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1647,47 +1605,31 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="27" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="24" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="27" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="24" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1695,7 +1637,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="29" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="26" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1703,15 +1645,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="29" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="26" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="19" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1719,11 +1661,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1731,11 +1673,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="19" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1743,15 +1685,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1759,67 +1701,67 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="36" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="39" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="39" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="40" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="41" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="42" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="41" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="41" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="45" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="42" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1839,7 +1781,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2471,11 +2413,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="24371910"/>
-        <c:axId val="67920695"/>
+        <c:axId val="85229886"/>
+        <c:axId val="24490517"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24371910"/>
+        <c:axId val="85229886"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2507,7 +2449,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67920695"/>
+        <c:crossAx val="24490517"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2515,7 +2457,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67920695"/>
+        <c:axId val="24490517"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2547,7 +2489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24371910"/>
+        <c:crossAx val="85229886"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2875,7 +2817,7 @@
     <tabColor rgb="FFCD212A"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3598,69 +3540,6 @@
       <c r="H35" s="22"/>
       <c r="I35" s="23"/>
       <c r="J35" s="24"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="D38" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" s="32" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C39" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="D39" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C39&amp;"*")</f>
-        <v>7</v>
-      </c>
-      <c r="E39" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C39&amp;"*",$E$11:$E$35,1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C40" s="33" t="s">
-        <v>89</v>
-      </c>
-      <c r="D40" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C40&amp;"*")</f>
-        <v>8</v>
-      </c>
-      <c r="E40" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C40&amp;"*",$E$11:$E$35,1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C41" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="D41" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C41&amp;"*")</f>
-        <v>7</v>
-      </c>
-      <c r="E41" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C41&amp;"*",$E$11:$E$35,1)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C42" s="33" t="s">
-        <v>90</v>
-      </c>
-      <c r="D42" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C42&amp;"*")</f>
-        <v>1</v>
-      </c>
-      <c r="E42" s="34" t="n">
-        <f aca="false">COUNTIFS($G$11:$G$35,"*"&amp;C42&amp;"*",$E$11:$E$35,1)</f>
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
   <autoFilter ref="A10:J35"/>
@@ -3756,7 +3635,7 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -3798,7 +3677,7 @@
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -3817,67 +3696,67 @@
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="N5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="35" t="n">
+      <c r="B6" s="31" t="n">
         <f aca="false">SUMIFS($J$11:$J$44,$M$11:$M$44,"Sì")</f>
         <v>4588.4</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36" t="n">
+      <c r="C6" s="31"/>
+      <c r="D6" s="32" t="n">
         <f aca="false">SUMIFS($J$11:$J$44,$L$11:$L$44,"Opzionale",$M$11:$M$44,"No")</f>
         <v>3000</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="E6" s="33" t="n">
         <f aca="false">B6+D6</f>
         <v>7588.4</v>
       </c>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="38" t="n">
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="34" t="n">
         <f aca="false">COUNTIFS($L$11:$L$44,"Da definire")</f>
         <v>7</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="39"/>
-      <c r="M6" s="40" t="str">
+      <c r="I6" s="34"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="36" t="str">
         <f aca="false">IF(J6="","",J6-B6)</f>
         <v/>
       </c>
-      <c r="N6" s="40"/>
+      <c r="N6" s="36"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3885,49 +3764,49 @@
         <v>10</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>14</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="L10" s="14" t="s">
         <v>17</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="O10" s="14" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="P10" s="14" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="Q10" s="15" t="s">
         <v>18</v>
@@ -3938,52 +3817,52 @@
         <v>1</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="E11" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="G11" s="43" t="n">
+        <v>109</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="G11" s="39" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I11" s="45" t="n">
+      <c r="H11" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I11" s="41" t="n">
         <f aca="false">180/100</f>
         <v>1.8</v>
       </c>
-      <c r="J11" s="46" t="n">
+      <c r="J11" s="42" t="n">
         <f aca="false">IF(OR(G11="",I11=""),"",G11*I11)</f>
         <v>180</v>
       </c>
-      <c r="K11" s="44" t="s">
-        <v>119</v>
+      <c r="K11" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L11" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M11" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N11" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O11" s="49"/>
-      <c r="P11" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M11" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N11" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O11" s="45"/>
+      <c r="P11" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q11" s="24" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3991,52 +3870,52 @@
         <v>2</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="41" t="s">
-        <v>127</v>
-      </c>
-      <c r="F12" s="42" t="s">
-        <v>128</v>
-      </c>
-      <c r="G12" s="43" t="n">
+        <v>120</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="39" t="n">
         <v>250</v>
       </c>
-      <c r="H12" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I12" s="45" t="n">
+      <c r="H12" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I12" s="41" t="n">
         <f aca="false">126/250</f>
         <v>0.504</v>
       </c>
-      <c r="J12" s="52" t="n">
+      <c r="J12" s="48" t="n">
         <f aca="false">IF(OR(G12="",I12=""),"",G12*I12)</f>
         <v>126</v>
       </c>
-      <c r="K12" s="51" t="s">
-        <v>119</v>
+      <c r="K12" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="M12" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="N12" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O12" s="49"/>
-      <c r="P12" s="50" t="s">
         <v>123</v>
       </c>
+      <c r="M12" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="N12" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O12" s="45"/>
+      <c r="P12" s="46" t="s">
+        <v>117</v>
+      </c>
       <c r="Q12" s="30" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4044,52 +3923,52 @@
         <v>3</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="E13" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="F13" s="42" t="s">
-        <v>128</v>
-      </c>
-      <c r="G13" s="43" t="n">
+      <c r="E13" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F13" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="G13" s="39" t="n">
         <v>250</v>
       </c>
-      <c r="H13" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I13" s="45" t="n">
+      <c r="H13" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I13" s="41" t="n">
         <f aca="false">50/250</f>
         <v>0.2</v>
       </c>
-      <c r="J13" s="46" t="n">
+      <c r="J13" s="42" t="n">
         <f aca="false">IF(OR(G13="",I13=""),"",G13*I13)</f>
         <v>50</v>
       </c>
-      <c r="K13" s="44" t="s">
-        <v>119</v>
+      <c r="K13" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M13" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N13" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O13" s="49"/>
-      <c r="P13" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M13" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N13" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O13" s="45"/>
+      <c r="P13" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q13" s="24" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4097,51 +3976,51 @@
         <v>4</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>136</v>
-      </c>
-      <c r="E14" s="41" t="s">
-        <v>137</v>
-      </c>
-      <c r="F14" s="42" t="s">
-        <v>138</v>
-      </c>
-      <c r="G14" s="43" t="n">
+        <v>130</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="F14" s="38" t="s">
+        <v>132</v>
+      </c>
+      <c r="G14" s="39" t="n">
         <v>200</v>
       </c>
-      <c r="H14" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I14" s="45" t="n">
+      <c r="H14" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I14" s="41" t="n">
         <v>1.2</v>
       </c>
-      <c r="J14" s="52" t="n">
+      <c r="J14" s="48" t="n">
         <f aca="false">IF(OR(G14="",I14=""),"",G14*I14)</f>
         <v>240</v>
       </c>
-      <c r="K14" s="51" t="s">
-        <v>119</v>
+      <c r="K14" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L14" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M14" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N14" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O14" s="49"/>
-      <c r="P14" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M14" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N14" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O14" s="45"/>
+      <c r="P14" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q14" s="30" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4149,48 +4028,48 @@
         <v>5</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="E15" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F15" s="42" t="s">
-        <v>144</v>
-      </c>
-      <c r="G15" s="43" t="n">
+        <v>136</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F15" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="G15" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I15" s="45" t="n">
+      <c r="H15" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I15" s="41" t="n">
         <v>37</v>
       </c>
-      <c r="J15" s="46" t="n">
+      <c r="J15" s="42" t="n">
         <f aca="false">IF(OR(G15="",I15=""),"",G15*I15)</f>
         <v>148</v>
       </c>
-      <c r="K15" s="44" t="s">
-        <v>119</v>
+      <c r="K15" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M15" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N15" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O15" s="49"/>
-      <c r="P15" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M15" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N15" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O15" s="45"/>
+      <c r="P15" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q15" s="24"/>
     </row>
@@ -4199,50 +4078,50 @@
         <v>6</v>
       </c>
       <c r="B16" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="E16" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F16" s="42" t="s">
-        <v>144</v>
-      </c>
-      <c r="G16" s="43" t="n">
+      <c r="E16" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F16" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="G16" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I16" s="45" t="n">
+      <c r="H16" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I16" s="41" t="n">
         <v>17.85</v>
       </c>
-      <c r="J16" s="52" t="n">
+      <c r="J16" s="48" t="n">
         <f aca="false">IF(OR(G16="",I16=""),"",G16*I16)</f>
         <v>71.4</v>
       </c>
-      <c r="K16" s="51" t="s">
-        <v>119</v>
+      <c r="K16" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M16" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N16" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O16" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="P16" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M16" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N16" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O16" s="45" t="s">
+        <v>141</v>
+      </c>
+      <c r="P16" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q16" s="30"/>
     </row>
@@ -4251,41 +4130,41 @@
         <v>7</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="E17" s="41"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="46" t="str">
+        <v>143</v>
+      </c>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="42" t="str">
         <f aca="false">IF(OR(G17="",I17=""),"",G17*I17)</f>
         <v/>
       </c>
-      <c r="K17" s="44" t="s">
-        <v>119</v>
+      <c r="K17" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L17" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="M17" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N17" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O17" s="49"/>
-      <c r="P17" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M17" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N17" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O17" s="45"/>
+      <c r="P17" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q17" s="24" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4293,52 +4172,52 @@
         <v>8</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>153</v>
-      </c>
-      <c r="E18" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F18" s="42"/>
-      <c r="G18" s="43" t="n">
+        <v>147</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F18" s="38"/>
+      <c r="G18" s="39" t="n">
         <v>6</v>
       </c>
-      <c r="H18" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I18" s="45" t="n">
+      <c r="H18" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I18" s="41" t="n">
         <f aca="false">130/6</f>
         <v>21.6666666666667</v>
       </c>
-      <c r="J18" s="52" t="n">
+      <c r="J18" s="48" t="n">
         <f aca="false">IF(OR(G18="",I18=""),"",G18*I18)</f>
         <v>130</v>
       </c>
-      <c r="K18" s="51" t="s">
-        <v>119</v>
+      <c r="K18" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L18" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M18" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N18" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O18" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="P18" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M18" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N18" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O18" s="45" t="s">
+        <v>148</v>
+      </c>
+      <c r="P18" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q18" s="30" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4346,45 +4225,45 @@
         <v>9</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="E19" s="41"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="43" t="n">
+        <v>152</v>
+      </c>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="H19" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I19" s="45"/>
-      <c r="J19" s="46" t="str">
+      <c r="H19" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I19" s="41"/>
+      <c r="J19" s="42" t="str">
         <f aca="false">IF(OR(G19="",I19=""),"",G19*I19)</f>
         <v/>
       </c>
-      <c r="K19" s="44" t="s">
-        <v>119</v>
+      <c r="K19" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L19" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="M19" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N19" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O19" s="49"/>
-      <c r="P19" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M19" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N19" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O19" s="45"/>
+      <c r="P19" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q19" s="24" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4392,48 +4271,48 @@
         <v>10</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="E20" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F20" s="42"/>
-      <c r="G20" s="43" t="n">
+        <v>155</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" s="38"/>
+      <c r="G20" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I20" s="45" t="n">
+      <c r="H20" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" s="41" t="n">
         <v>60</v>
       </c>
-      <c r="J20" s="52" t="n">
+      <c r="J20" s="48" t="n">
         <f aca="false">IF(OR(G20="",I20=""),"",G20*I20)</f>
         <v>60</v>
       </c>
-      <c r="K20" s="51" t="s">
-        <v>119</v>
+      <c r="K20" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L20" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M20" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N20" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O20" s="49" t="s">
-        <v>162</v>
-      </c>
-      <c r="P20" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M20" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N20" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O20" s="45" t="s">
+        <v>156</v>
+      </c>
+      <c r="P20" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q20" s="30"/>
     </row>
@@ -4442,48 +4321,48 @@
         <v>11</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="E21" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F21" s="42"/>
-      <c r="G21" s="43" t="n">
+        <v>158</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F21" s="38"/>
+      <c r="G21" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I21" s="45" t="n">
+      <c r="H21" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I21" s="41" t="n">
         <v>60</v>
       </c>
-      <c r="J21" s="46" t="n">
+      <c r="J21" s="42" t="n">
         <f aca="false">IF(OR(G21="",I21=""),"",G21*I21)</f>
         <v>60</v>
       </c>
-      <c r="K21" s="44" t="s">
-        <v>119</v>
+      <c r="K21" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L21" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M21" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N21" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O21" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="P21" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M21" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N21" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O21" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="P21" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q21" s="24"/>
     </row>
@@ -4492,51 +4371,51 @@
         <v>12</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>167</v>
-      </c>
-      <c r="E22" s="41" t="s">
-        <v>168</v>
-      </c>
-      <c r="F22" s="42"/>
-      <c r="G22" s="43" t="n">
+        <v>161</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="F22" s="38"/>
+      <c r="G22" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="51" t="s">
-        <v>169</v>
-      </c>
-      <c r="I22" s="45" t="n">
+      <c r="H22" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="I22" s="41" t="n">
         <v>390</v>
       </c>
-      <c r="J22" s="52" t="n">
+      <c r="J22" s="48" t="n">
         <f aca="false">IF(OR(G22="",I22=""),"",G22*I22)</f>
         <v>390</v>
       </c>
-      <c r="K22" s="51" t="s">
-        <v>119</v>
+      <c r="K22" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L22" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M22" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N22" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O22" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="P22" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M22" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N22" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O22" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="P22" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q22" s="30" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4544,48 +4423,48 @@
         <v>13</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="E23" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="F23" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="G23" s="43" t="n">
+        <v>166</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" s="39" t="n">
         <v>18</v>
       </c>
-      <c r="H23" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I23" s="45" t="n">
+      <c r="H23" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I23" s="41" t="n">
         <v>54</v>
       </c>
-      <c r="J23" s="46" t="n">
+      <c r="J23" s="42" t="n">
         <f aca="false">IF(OR(G23="",I23=""),"",G23*I23)</f>
         <v>972</v>
       </c>
-      <c r="K23" s="44" t="s">
-        <v>173</v>
+      <c r="K23" s="40" t="s">
+        <v>167</v>
       </c>
       <c r="L23" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M23" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N23" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O23" s="49"/>
-      <c r="P23" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M23" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N23" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O23" s="45"/>
+      <c r="P23" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q23" s="24"/>
     </row>
@@ -4594,50 +4473,50 @@
         <v>14</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>175</v>
-      </c>
-      <c r="E24" s="41" t="s">
-        <v>127</v>
-      </c>
-      <c r="F24" s="42"/>
-      <c r="G24" s="43" t="n">
+        <v>169</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F24" s="38"/>
+      <c r="G24" s="39" t="n">
         <v>18</v>
       </c>
-      <c r="H24" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I24" s="45" t="n">
+      <c r="H24" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I24" s="41" t="n">
         <f aca="false">654/18</f>
         <v>36.3333333333333</v>
       </c>
-      <c r="J24" s="52" t="n">
+      <c r="J24" s="48" t="n">
         <f aca="false">IF(OR(G24="",I24=""),"",G24*I24)</f>
         <v>654</v>
       </c>
-      <c r="K24" s="51" t="s">
-        <v>119</v>
+      <c r="K24" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L24" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="M24" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="N24" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O24" s="49"/>
-      <c r="P24" s="50" t="s">
         <v>123</v>
       </c>
+      <c r="M24" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="N24" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O24" s="45"/>
+      <c r="P24" s="46" t="s">
+        <v>117</v>
+      </c>
       <c r="Q24" s="30" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4645,49 +4524,49 @@
         <v>15</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="E25" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="F25" s="42"/>
-      <c r="G25" s="43" t="n">
+        <v>172</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F25" s="38"/>
+      <c r="G25" s="39" t="n">
         <v>13</v>
       </c>
-      <c r="H25" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I25" s="45" t="n">
+      <c r="H25" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="J25" s="46" t="n">
+      <c r="J25" s="42" t="n">
         <f aca="false">IF(OR(G25="",I25=""),"",G25*I25)</f>
         <v>52</v>
       </c>
-      <c r="K25" s="44" t="s">
+      <c r="K25" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="L25" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="M25" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N25" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O25" s="45"/>
+      <c r="P25" s="46" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q25" s="24" t="s">
         <v>173</v>
-      </c>
-      <c r="L25" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M25" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N25" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O25" s="49"/>
-      <c r="P25" s="50" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q25" s="24" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4695,45 +4574,45 @@
         <v>16</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="E26" s="41" t="s">
-        <v>127</v>
-      </c>
-      <c r="F26" s="42"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I26" s="45"/>
-      <c r="J26" s="52" t="str">
+        <v>175</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F26" s="38"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I26" s="41"/>
+      <c r="J26" s="48" t="str">
         <f aca="false">IF(OR(G26="",I26=""),"",G26*I26)</f>
         <v/>
       </c>
-      <c r="K26" s="51" t="s">
-        <v>119</v>
+      <c r="K26" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L26" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="M26" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N26" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O26" s="49"/>
-      <c r="P26" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M26" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N26" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O26" s="45"/>
+      <c r="P26" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q26" s="30" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4741,49 +4620,49 @@
         <v>17</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="E27" s="41" t="s">
-        <v>127</v>
-      </c>
-      <c r="F27" s="42"/>
-      <c r="G27" s="43" t="n">
+        <v>178</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F27" s="38"/>
+      <c r="G27" s="39" t="n">
         <v>18</v>
       </c>
-      <c r="H27" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I27" s="45" t="n">
+      <c r="H27" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I27" s="41" t="n">
         <v>125</v>
       </c>
-      <c r="J27" s="46" t="n">
+      <c r="J27" s="42" t="n">
         <f aca="false">IF(OR(G27="",I27=""),"",G27*I27)</f>
         <v>2250</v>
       </c>
-      <c r="K27" s="44" t="s">
-        <v>119</v>
+      <c r="K27" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L27" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="M27" s="47" t="s">
-        <v>130</v>
-      </c>
-      <c r="N27" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O27" s="49"/>
-      <c r="P27" s="50" t="s">
-        <v>123</v>
+        <v>179</v>
+      </c>
+      <c r="M27" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="N27" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O27" s="45"/>
+      <c r="P27" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q27" s="24" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4791,48 +4670,48 @@
         <v>18</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>188</v>
-      </c>
-      <c r="E28" s="41"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="43" t="n">
+        <v>182</v>
+      </c>
+      <c r="E28" s="37"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="51" t="s">
-        <v>169</v>
-      </c>
-      <c r="I28" s="45" t="n">
+      <c r="H28" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="I28" s="41" t="n">
         <f aca="false">150/1</f>
         <v>150</v>
       </c>
-      <c r="J28" s="52" t="n">
+      <c r="J28" s="48" t="n">
         <f aca="false">IF(OR(G28="",I28=""),"",G28*I28)</f>
         <v>150</v>
       </c>
-      <c r="K28" s="51" t="s">
-        <v>119</v>
+      <c r="K28" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L28" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="M28" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="N28" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O28" s="49"/>
-      <c r="P28" s="50" t="s">
-        <v>123</v>
+        <v>179</v>
+      </c>
+      <c r="M28" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="N28" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O28" s="45"/>
+      <c r="P28" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q28" s="30" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4840,46 +4719,46 @@
         <v>19</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="E29" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="F29" s="42"/>
-      <c r="G29" s="43" t="n">
+        <v>186</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F29" s="38"/>
+      <c r="G29" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I29" s="45" t="n">
+      <c r="H29" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I29" s="41" t="n">
         <v>85</v>
       </c>
-      <c r="J29" s="46" t="n">
+      <c r="J29" s="42" t="n">
         <f aca="false">IF(OR(G29="",I29=""),"",G29*I29)</f>
         <v>85</v>
       </c>
-      <c r="K29" s="44" t="s">
-        <v>173</v>
+      <c r="K29" s="40" t="s">
+        <v>167</v>
       </c>
       <c r="L29" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M29" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N29" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O29" s="49"/>
-      <c r="P29" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M29" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N29" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O29" s="45"/>
+      <c r="P29" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q29" s="24"/>
     </row>
@@ -4888,46 +4767,46 @@
         <v>20</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="E30" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F30" s="42"/>
-      <c r="G30" s="43" t="n">
+        <v>188</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F30" s="38"/>
+      <c r="G30" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I30" s="45" t="n">
+      <c r="H30" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I30" s="41" t="n">
         <v>80</v>
       </c>
-      <c r="J30" s="52" t="n">
+      <c r="J30" s="48" t="n">
         <f aca="false">IF(OR(G30="",I30=""),"",G30*I30)</f>
         <v>80</v>
       </c>
-      <c r="K30" s="51" t="s">
-        <v>119</v>
+      <c r="K30" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L30" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M30" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N30" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O30" s="49"/>
-      <c r="P30" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M30" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N30" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O30" s="45"/>
+      <c r="P30" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q30" s="30"/>
     </row>
@@ -4936,47 +4815,47 @@
         <v>21</v>
       </c>
       <c r="B31" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="D31" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>196</v>
-      </c>
-      <c r="E31" s="41"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="43" t="n">
+      <c r="E31" s="37"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H31" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I31" s="45" t="n">
+      <c r="H31" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I31" s="41" t="n">
         <v>600</v>
       </c>
-      <c r="J31" s="46" t="n">
+      <c r="J31" s="42" t="n">
         <f aca="false">IF(OR(G31="",I31=""),"",G31*I31)</f>
         <v>600</v>
       </c>
-      <c r="K31" s="44" t="s">
-        <v>119</v>
+      <c r="K31" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L31" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="M31" s="47" t="s">
-        <v>130</v>
-      </c>
-      <c r="N31" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O31" s="49"/>
-      <c r="P31" s="50" t="s">
-        <v>123</v>
+        <v>179</v>
+      </c>
+      <c r="M31" s="43" t="s">
+        <v>124</v>
+      </c>
+      <c r="N31" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O31" s="45"/>
+      <c r="P31" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q31" s="24" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4984,47 +4863,47 @@
         <v>22</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D32" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="E32" s="41"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="43" t="n">
+        <v>193</v>
+      </c>
+      <c r="E32" s="37"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="H32" s="51" t="s">
-        <v>200</v>
-      </c>
-      <c r="I32" s="45" t="n">
+      <c r="H32" s="47" t="s">
+        <v>194</v>
+      </c>
+      <c r="I32" s="41" t="n">
         <v>150</v>
       </c>
-      <c r="J32" s="52" t="n">
+      <c r="J32" s="48" t="n">
         <f aca="false">IF(OR(G32="",I32=""),"",G32*I32)</f>
         <v>300</v>
       </c>
-      <c r="K32" s="51" t="s">
-        <v>119</v>
+      <c r="K32" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>201</v>
-      </c>
-      <c r="M32" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N32" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O32" s="49"/>
-      <c r="P32" s="50" t="s">
-        <v>123</v>
+        <v>195</v>
+      </c>
+      <c r="M32" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N32" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O32" s="45"/>
+      <c r="P32" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q32" s="30" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5032,45 +4911,45 @@
         <v>23</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="E33" s="41"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="43" t="n">
+        <v>198</v>
+      </c>
+      <c r="E33" s="37"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I33" s="45"/>
-      <c r="J33" s="46" t="str">
+      <c r="H33" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I33" s="41"/>
+      <c r="J33" s="42" t="str">
         <f aca="false">IF(OR(G33="",I33=""),"",G33*I33)</f>
         <v/>
       </c>
-      <c r="K33" s="44" t="s">
-        <v>119</v>
+      <c r="K33" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L33" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="M33" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N33" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O33" s="49"/>
-      <c r="P33" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M33" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N33" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O33" s="45"/>
+      <c r="P33" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q33" s="24" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5078,45 +4957,45 @@
         <v>24</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="E34" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="F34" s="42"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="I34" s="45"/>
-      <c r="J34" s="52" t="str">
+        <v>202</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="F34" s="38"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="I34" s="41"/>
+      <c r="J34" s="48" t="str">
         <f aca="false">IF(OR(G34="",I34=""),"",G34*I34)</f>
         <v/>
       </c>
-      <c r="K34" s="51" t="s">
-        <v>119</v>
+      <c r="K34" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L34" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="M34" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N34" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O34" s="49"/>
-      <c r="P34" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M34" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N34" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O34" s="45"/>
+      <c r="P34" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q34" s="30" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5124,50 +5003,50 @@
         <v>25</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="E35" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="F35" s="42"/>
-      <c r="G35" s="43" t="n">
+        <v>205</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F35" s="38"/>
+      <c r="G35" s="39" t="n">
         <v>100</v>
       </c>
-      <c r="H35" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="I35" s="45" t="n">
+      <c r="H35" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="I35" s="41" t="n">
         <f aca="false">370/100</f>
         <v>3.7</v>
       </c>
-      <c r="J35" s="46" t="n">
+      <c r="J35" s="42" t="n">
         <f aca="false">IF(OR(G35="",I35=""),"",G35*I35)</f>
         <v>370</v>
       </c>
-      <c r="K35" s="44" t="s">
-        <v>173</v>
+      <c r="K35" s="40" t="s">
+        <v>167</v>
       </c>
       <c r="L35" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="M35" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N35" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O35" s="49"/>
-      <c r="P35" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M35" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N35" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O35" s="45"/>
+      <c r="P35" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q35" s="24" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5175,46 +5054,46 @@
         <v>26</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D36" s="28" t="s">
-        <v>214</v>
-      </c>
-      <c r="E36" s="41" t="s">
-        <v>215</v>
-      </c>
-      <c r="F36" s="42"/>
-      <c r="G36" s="43" t="n">
+        <v>208</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="F36" s="38"/>
+      <c r="G36" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H36" s="51" t="s">
-        <v>216</v>
-      </c>
-      <c r="I36" s="45" t="n">
+      <c r="H36" s="47" t="s">
+        <v>210</v>
+      </c>
+      <c r="I36" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="J36" s="52" t="n">
+      <c r="J36" s="48" t="n">
         <f aca="false">IF(OR(G36="",I36=""),"",G36*I36)</f>
         <v>300</v>
       </c>
-      <c r="K36" s="51" t="s">
-        <v>119</v>
+      <c r="K36" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L36" s="29" t="s">
-        <v>120</v>
-      </c>
-      <c r="M36" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N36" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O36" s="49"/>
-      <c r="P36" s="50" t="s">
-        <v>123</v>
+        <v>114</v>
+      </c>
+      <c r="M36" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N36" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O36" s="45"/>
+      <c r="P36" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q36" s="30"/>
     </row>
@@ -5223,45 +5102,45 @@
         <v>27</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="E37" s="41"/>
-      <c r="F37" s="42" t="s">
+        <v>213</v>
+      </c>
+      <c r="E37" s="37"/>
+      <c r="F37" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44" t="s">
-        <v>220</v>
-      </c>
-      <c r="I37" s="45"/>
-      <c r="J37" s="46" t="str">
+      <c r="G37" s="39"/>
+      <c r="H37" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="I37" s="41"/>
+      <c r="J37" s="42" t="str">
         <f aca="false">IF(OR(G37="",I37=""),"",G37*I37)</f>
         <v/>
       </c>
-      <c r="K37" s="44" t="s">
-        <v>119</v>
+      <c r="K37" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L37" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="M37" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N37" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O37" s="49"/>
-      <c r="P37" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M37" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N37" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O37" s="45"/>
+      <c r="P37" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q37" s="24" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5269,7 +5148,7 @@
         <v>28</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C38" s="27" t="s">
         <v>76</v>
@@ -5277,40 +5156,40 @@
       <c r="D38" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="E38" s="41"/>
-      <c r="F38" s="42"/>
-      <c r="G38" s="43" t="n">
+      <c r="E38" s="37"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H38" s="51" t="s">
-        <v>222</v>
-      </c>
-      <c r="I38" s="45" t="n">
+      <c r="H38" s="47" t="s">
+        <v>216</v>
+      </c>
+      <c r="I38" s="41" t="n">
         <f aca="false">1100/1</f>
         <v>1100</v>
       </c>
-      <c r="J38" s="52" t="n">
+      <c r="J38" s="48" t="n">
         <f aca="false">IF(OR(G38="",I38=""),"",G38*I38)</f>
         <v>1100</v>
       </c>
-      <c r="K38" s="51" t="s">
-        <v>119</v>
+      <c r="K38" s="47" t="s">
+        <v>113</v>
       </c>
       <c r="L38" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="M38" s="53" t="s">
-        <v>121</v>
-      </c>
-      <c r="N38" s="54" t="s">
-        <v>122</v>
-      </c>
-      <c r="O38" s="49"/>
-      <c r="P38" s="50" t="s">
-        <v>123</v>
+        <v>217</v>
+      </c>
+      <c r="M38" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="N38" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="O38" s="45"/>
+      <c r="P38" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q38" s="30" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5318,43 +5197,43 @@
         <v>29</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="E39" s="41"/>
-      <c r="F39" s="42"/>
-      <c r="G39" s="43"/>
-      <c r="H39" s="44" t="s">
-        <v>227</v>
-      </c>
-      <c r="I39" s="45"/>
-      <c r="J39" s="46" t="str">
+        <v>220</v>
+      </c>
+      <c r="E39" s="37"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="39"/>
+      <c r="H39" s="40" t="s">
+        <v>221</v>
+      </c>
+      <c r="I39" s="41"/>
+      <c r="J39" s="42" t="str">
         <f aca="false">IF(OR(G39="",I39=""),"",G39*I39)</f>
         <v/>
       </c>
-      <c r="K39" s="44" t="s">
-        <v>119</v>
+      <c r="K39" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="L39" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="M39" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="N39" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="O39" s="49"/>
-      <c r="P39" s="50" t="s">
-        <v>123</v>
+        <v>144</v>
+      </c>
+      <c r="M39" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="N39" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="O39" s="45"/>
+      <c r="P39" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q39" s="24" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5364,22 +5243,22 @@
       <c r="B40" s="26"/>
       <c r="C40" s="27"/>
       <c r="D40" s="28"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="42"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="51"/>
-      <c r="I40" s="45"/>
-      <c r="J40" s="52" t="str">
+      <c r="E40" s="37"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="39"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="41"/>
+      <c r="J40" s="48" t="str">
         <f aca="false">IF(OR(G40="",I40=""),"",G40*I40)</f>
         <v/>
       </c>
-      <c r="K40" s="51"/>
+      <c r="K40" s="47"/>
       <c r="L40" s="29"/>
-      <c r="M40" s="53"/>
-      <c r="N40" s="54"/>
-      <c r="O40" s="49"/>
-      <c r="P40" s="50" t="s">
-        <v>123</v>
+      <c r="M40" s="49"/>
+      <c r="N40" s="50"/>
+      <c r="O40" s="45"/>
+      <c r="P40" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q40" s="30"/>
     </row>
@@ -5390,22 +5269,22 @@
       <c r="B41" s="17"/>
       <c r="C41" s="18"/>
       <c r="D41" s="19"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="42"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="46" t="str">
+      <c r="E41" s="37"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="39"/>
+      <c r="H41" s="40"/>
+      <c r="I41" s="41"/>
+      <c r="J41" s="42" t="str">
         <f aca="false">IF(OR(G41="",I41=""),"",G41*I41)</f>
         <v/>
       </c>
-      <c r="K41" s="44"/>
+      <c r="K41" s="40"/>
       <c r="L41" s="23"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="48"/>
-      <c r="O41" s="49"/>
-      <c r="P41" s="50" t="s">
-        <v>123</v>
+      <c r="M41" s="43"/>
+      <c r="N41" s="44"/>
+      <c r="O41" s="45"/>
+      <c r="P41" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q41" s="24"/>
     </row>
@@ -5416,22 +5295,22 @@
       <c r="B42" s="26"/>
       <c r="C42" s="27"/>
       <c r="D42" s="28"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="43"/>
-      <c r="H42" s="51"/>
-      <c r="I42" s="45"/>
-      <c r="J42" s="52" t="str">
+      <c r="E42" s="37"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="39"/>
+      <c r="H42" s="47"/>
+      <c r="I42" s="41"/>
+      <c r="J42" s="48" t="str">
         <f aca="false">IF(OR(G42="",I42=""),"",G42*I42)</f>
         <v/>
       </c>
-      <c r="K42" s="51"/>
+      <c r="K42" s="47"/>
       <c r="L42" s="29"/>
-      <c r="M42" s="53"/>
-      <c r="N42" s="54"/>
-      <c r="O42" s="49"/>
-      <c r="P42" s="50" t="s">
-        <v>123</v>
+      <c r="M42" s="49"/>
+      <c r="N42" s="50"/>
+      <c r="O42" s="45"/>
+      <c r="P42" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q42" s="30"/>
     </row>
@@ -5442,22 +5321,22 @@
       <c r="B43" s="17"/>
       <c r="C43" s="18"/>
       <c r="D43" s="19"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="42"/>
-      <c r="G43" s="43"/>
-      <c r="H43" s="44"/>
-      <c r="I43" s="45"/>
-      <c r="J43" s="46" t="str">
+      <c r="E43" s="37"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="39"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="41"/>
+      <c r="J43" s="42" t="str">
         <f aca="false">IF(OR(G43="",I43=""),"",G43*I43)</f>
         <v/>
       </c>
-      <c r="K43" s="44"/>
+      <c r="K43" s="40"/>
       <c r="L43" s="23"/>
-      <c r="M43" s="47"/>
-      <c r="N43" s="48"/>
-      <c r="O43" s="49"/>
-      <c r="P43" s="50" t="s">
-        <v>123</v>
+      <c r="M43" s="43"/>
+      <c r="N43" s="44"/>
+      <c r="O43" s="45"/>
+      <c r="P43" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q43" s="24"/>
     </row>
@@ -5468,30 +5347,30 @@
       <c r="B44" s="26"/>
       <c r="C44" s="27"/>
       <c r="D44" s="28"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="42"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="51"/>
-      <c r="I44" s="45"/>
-      <c r="J44" s="52" t="str">
+      <c r="E44" s="37"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="39"/>
+      <c r="H44" s="47"/>
+      <c r="I44" s="41"/>
+      <c r="J44" s="48" t="str">
         <f aca="false">IF(OR(G44="",I44=""),"",G44*I44)</f>
         <v/>
       </c>
-      <c r="K44" s="51"/>
+      <c r="K44" s="47"/>
       <c r="L44" s="29"/>
-      <c r="M44" s="53"/>
-      <c r="N44" s="54"/>
-      <c r="O44" s="49"/>
-      <c r="P44" s="50" t="s">
-        <v>123</v>
+      <c r="M44" s="49"/>
+      <c r="N44" s="50"/>
+      <c r="O44" s="45"/>
+      <c r="P44" s="46" t="s">
+        <v>117</v>
       </c>
       <c r="Q44" s="30"/>
     </row>
     <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
-      <c r="C45" s="55" t="s">
-        <v>229</v>
+      <c r="C45" s="51" t="s">
+        <v>223</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -5499,7 +5378,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
-      <c r="J45" s="56" t="n">
+      <c r="J45" s="52" t="n">
         <f aca="false">SUMIFS($J$11:$J$44,$M$11:$M$44,"Sì")</f>
         <v>4588.4</v>
       </c>
@@ -5512,28 +5391,28 @@
       <c r="Q45" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="57" t="s">
-        <v>230</v>
+      <c r="B47" s="53" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="58" t="s">
-        <v>231</v>
+      <c r="B48" s="54" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="58" t="s">
-        <v>232</v>
+      <c r="B49" s="54" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="58" t="s">
-        <v>233</v>
+      <c r="B50" s="54" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="58" t="s">
-        <v>234</v>
+      <c r="B51" s="54" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -5637,8 +5516,8 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="59" t="s">
-        <v>235</v>
+      <c r="B1" s="55" t="s">
+        <v>229</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -5648,8 +5527,8 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
-      <c r="B2" s="60" t="s">
-        <v>236</v>
+      <c r="B2" s="56" t="s">
+        <v>230</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5658,216 +5537,216 @@
       <c r="G2" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="61"/>
-      <c r="B4" s="62" t="s">
-        <v>100</v>
-      </c>
-      <c r="C4" s="61" t="s">
-        <v>237</v>
-      </c>
-      <c r="D4" s="61" t="s">
-        <v>93</v>
-      </c>
-      <c r="E4" s="61" t="s">
+      <c r="A4" s="57"/>
+      <c r="B4" s="58" t="s">
         <v>94</v>
       </c>
-      <c r="F4" s="61" t="s">
-        <v>107</v>
-      </c>
-      <c r="G4" s="61" t="s">
-        <v>238</v>
+      <c r="C4" s="57" t="s">
+        <v>231</v>
+      </c>
+      <c r="D4" s="57" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="57" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="57" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="57" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="63" t="s">
-        <v>239</v>
-      </c>
-      <c r="B5" s="64" t="s">
-        <v>240</v>
-      </c>
-      <c r="C5" s="65" t="n">
+      <c r="A5" s="59" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="60" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"A · Materiale marketing")</f>
         <v>4</v>
       </c>
-      <c r="D5" s="66" t="n">
+      <c r="D5" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"A · Materiale marketing",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>470</v>
       </c>
-      <c r="E5" s="67" t="n">
+      <c r="E5" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"A · Materiale marketing",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="67" t="n">
+      <c r="F5" s="63" t="n">
         <f aca="false">D5+E5</f>
         <v>470</v>
       </c>
-      <c r="G5" s="68" t="n">
+      <c r="G5" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D5/$D$11)</f>
         <v>0.102432220381832</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="63" t="s">
-        <v>241</v>
-      </c>
-      <c r="B6" s="64" t="s">
-        <v>242</v>
-      </c>
-      <c r="C6" s="65" t="n">
+      <c r="A6" s="59" t="s">
+        <v>235</v>
+      </c>
+      <c r="B6" s="60" t="s">
+        <v>236</v>
+      </c>
+      <c r="C6" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"B · Punto ristoro e briefing")</f>
         <v>4</v>
       </c>
-      <c r="D6" s="66" t="n">
+      <c r="D6" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"B · Punto ristoro e briefing",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>349.4</v>
       </c>
-      <c r="E6" s="67" t="n">
+      <c r="E6" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"B · Punto ristoro e briefing",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="67" t="n">
+      <c r="F6" s="63" t="n">
         <f aca="false">D6+E6</f>
         <v>349.4</v>
       </c>
-      <c r="G6" s="68" t="n">
+      <c r="G6" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D6/$D$11)</f>
         <v>0.0761485485136431</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="63" t="s">
-        <v>243</v>
-      </c>
-      <c r="B7" s="64" t="s">
-        <v>244</v>
-      </c>
-      <c r="C7" s="65" t="n">
+      <c r="A7" s="59" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C7" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"C · Percorso e partenze")</f>
         <v>10</v>
       </c>
-      <c r="D7" s="66" t="n">
+      <c r="D7" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"C · Percorso e partenze",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>1534</v>
       </c>
-      <c r="E7" s="67" t="n">
+      <c r="E7" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"C · Percorso e partenze",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>2400</v>
       </c>
-      <c r="F7" s="67" t="n">
+      <c r="F7" s="63" t="n">
         <f aca="false">D7+E7</f>
         <v>3934</v>
       </c>
-      <c r="G7" s="68" t="n">
+      <c r="G7" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D7/$D$11)</f>
         <v>0.334321332054747</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="63" t="s">
-        <v>245</v>
-      </c>
-      <c r="B8" s="64" t="s">
-        <v>246</v>
-      </c>
-      <c r="C8" s="65" t="n">
+      <c r="A8" s="59" t="s">
+        <v>239</v>
+      </c>
+      <c r="B8" s="60" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"D · Immagine e media")</f>
         <v>5</v>
       </c>
-      <c r="D8" s="66" t="n">
+      <c r="D8" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"D · Immagine e media",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>465</v>
       </c>
-      <c r="E8" s="67" t="n">
+      <c r="E8" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"D · Immagine e media",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>600</v>
       </c>
-      <c r="F8" s="67" t="n">
+      <c r="F8" s="63" t="n">
         <f aca="false">D8+E8</f>
         <v>1065</v>
       </c>
-      <c r="G8" s="68" t="n">
+      <c r="G8" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D8/$D$11)</f>
         <v>0.101342515909685</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="63" t="s">
-        <v>247</v>
-      </c>
-      <c r="B9" s="64" t="s">
-        <v>248</v>
-      </c>
-      <c r="C9" s="65" t="n">
+      <c r="A9" s="59" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>242</v>
+      </c>
+      <c r="C9" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"E · Accoglienza")</f>
         <v>3</v>
       </c>
-      <c r="D9" s="66" t="n">
+      <c r="D9" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"E · Accoglienza",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>670</v>
       </c>
-      <c r="E9" s="67" t="n">
+      <c r="E9" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"E · Accoglienza",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="67" t="n">
+      <c r="F9" s="63" t="n">
         <f aca="false">D9+E9</f>
         <v>670</v>
       </c>
-      <c r="G9" s="68" t="n">
+      <c r="G9" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D9/$D$11)</f>
         <v>0.146020399267719</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="63" t="s">
-        <v>249</v>
-      </c>
-      <c r="B10" s="64" t="s">
-        <v>250</v>
-      </c>
-      <c r="C10" s="65" t="n">
+      <c r="A10" s="59" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" s="60" t="s">
+        <v>244</v>
+      </c>
+      <c r="C10" s="61" t="n">
         <f aca="false">COUNTIFS(Preventivo!$B$11:$B$44,"F · Staff e ospitalità")</f>
         <v>3</v>
       </c>
-      <c r="D10" s="66" t="n">
+      <c r="D10" s="62" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"F · Staff e ospitalità",Preventivo!$M$11:$M$44,"Sì")</f>
         <v>1100</v>
       </c>
-      <c r="E10" s="67" t="n">
+      <c r="E10" s="63" t="n">
         <f aca="false">SUMIFS(Preventivo!$J$11:$J$44,Preventivo!$B$11:$B$44,"F · Staff e ospitalità",Preventivo!$L$11:$L$44,"Opzionale",Preventivo!$M$11:$M$44,"No")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="67" t="n">
+      <c r="F10" s="63" t="n">
         <f aca="false">D10+E10</f>
         <v>1100</v>
       </c>
-      <c r="G10" s="68" t="n">
+      <c r="G10" s="64" t="n">
         <f aca="false">IF($D$11=0,0,D10/$D$11)</f>
         <v>0.239734983872374</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="B11" s="69" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" s="70" t="n">
+      <c r="B11" s="65" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="66" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>29</v>
       </c>
-      <c r="D11" s="71" t="n">
+      <c r="D11" s="67" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>4588.4</v>
       </c>
-      <c r="E11" s="72" t="n">
+      <c r="E11" s="68" t="n">
         <f aca="false">SUM(E5:E10)</f>
         <v>3000</v>
       </c>
-      <c r="F11" s="72" t="n">
+      <c r="F11" s="68" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>7588.4</v>
       </c>
-      <c r="G11" s="73" t="n">
+      <c r="G11" s="69" t="n">
         <f aca="false">IF($D$11=0,0,SUM(G5:G10))</f>
         <v>1</v>
       </c>
@@ -5901,175 +5780,175 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="74" t="s">
-        <v>251</v>
+      <c r="B1" s="70" t="s">
+        <v>245</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
-      <c r="B2" s="60" t="s">
-        <v>252</v>
+      <c r="B2" s="56" t="s">
+        <v>246</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75" t="s">
+      <c r="A4" s="71"/>
+      <c r="B4" s="71" t="s">
+        <v>247</v>
+      </c>
+      <c r="C4" s="71" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4" s="71" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="72"/>
+      <c r="B5" s="73" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" s="72"/>
+      <c r="D5" s="74"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="72"/>
+      <c r="B6" s="73" t="s">
+        <v>251</v>
+      </c>
+      <c r="C6" s="72"/>
+      <c r="D6" s="74"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="72"/>
+      <c r="B7" s="73" t="s">
+        <v>252</v>
+      </c>
+      <c r="C7" s="72"/>
+      <c r="D7" s="74"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="75" t="s">
         <v>253</v>
       </c>
-      <c r="C4" s="75" t="s">
+      <c r="D8" s="76"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="75" t="s">
         <v>254</v>
       </c>
-      <c r="D4" s="75" t="s">
+      <c r="D9" s="76"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="75" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="76"/>
-      <c r="B5" s="77" t="s">
+      <c r="D10" s="76"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="75" t="s">
         <v>256</v>
       </c>
-      <c r="C5" s="76"/>
-      <c r="D5" s="78"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="76"/>
-      <c r="B6" s="77" t="s">
+      <c r="D11" s="76"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="72"/>
+      <c r="B12" s="73" t="s">
         <v>257</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="78"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="76"/>
-      <c r="B7" s="77" t="s">
+      <c r="C12" s="72"/>
+      <c r="D12" s="74"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="75" t="s">
         <v>258</v>
       </c>
-      <c r="C7" s="76"/>
-      <c r="D7" s="78"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="79" t="s">
+      <c r="D13" s="76"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="75" t="s">
         <v>259</v>
       </c>
-      <c r="D8" s="80"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C9" s="79" t="s">
+      <c r="D14" s="76"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="D9" s="80"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="79" t="s">
+      <c r="D15" s="76"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="72"/>
+      <c r="B16" s="73" t="s">
         <v>261</v>
       </c>
-      <c r="D10" s="80"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="79" t="s">
+      <c r="C16" s="72"/>
+      <c r="D16" s="74"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="72"/>
+      <c r="B17" s="73" t="s">
         <v>262</v>
       </c>
-      <c r="D11" s="80"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="76"/>
-      <c r="B12" s="77" t="s">
+      <c r="C17" s="72"/>
+      <c r="D17" s="74"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="75" t="s">
         <v>263</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="78"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="79" t="s">
+      <c r="D18" s="76"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="75" t="s">
         <v>264</v>
       </c>
-      <c r="D13" s="80"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="79" t="s">
+      <c r="D19" s="76"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="75" t="s">
         <v>265</v>
       </c>
-      <c r="D14" s="80"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="79" t="s">
+      <c r="D20" s="76"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="75" t="s">
         <v>266</v>
       </c>
-      <c r="D15" s="80"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="76"/>
-      <c r="B16" s="77" t="s">
+      <c r="D21" s="76"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="75" t="s">
         <v>267</v>
       </c>
-      <c r="C16" s="76"/>
-      <c r="D16" s="78"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="76"/>
-      <c r="B17" s="77" t="s">
+      <c r="D22" s="76"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="72"/>
+      <c r="B23" s="73" t="s">
         <v>268</v>
       </c>
-      <c r="C17" s="76"/>
-      <c r="D17" s="78"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="79" t="s">
+      <c r="C23" s="72"/>
+      <c r="D23" s="74"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="72"/>
+      <c r="B24" s="73" t="s">
         <v>269</v>
       </c>
-      <c r="D18" s="80"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="79" t="s">
+      <c r="C24" s="72"/>
+      <c r="D24" s="74"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="72"/>
+      <c r="B25" s="73" t="s">
         <v>270</v>
       </c>
-      <c r="D19" s="80"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="79" t="s">
-        <v>271</v>
-      </c>
-      <c r="D20" s="80"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="79" t="s">
-        <v>272</v>
-      </c>
-      <c r="D21" s="80"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="79" t="s">
-        <v>273</v>
-      </c>
-      <c r="D22" s="80"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="76"/>
-      <c r="B23" s="77" t="s">
-        <v>274</v>
-      </c>
-      <c r="C23" s="76"/>
-      <c r="D23" s="78"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="76"/>
-      <c r="B24" s="77" t="s">
-        <v>275</v>
-      </c>
-      <c r="C24" s="76"/>
-      <c r="D24" s="78"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="76"/>
-      <c r="B25" s="77" t="s">
-        <v>276</v>
-      </c>
-      <c r="C25" s="76"/>
-      <c r="D25" s="78"/>
+      <c r="C25" s="72"/>
+      <c r="D25" s="74"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>